<commit_message>
fixed string output thing
</commit_message>
<xml_diff>
--- a/Astra Notes.xlsx
+++ b/Astra Notes.xlsx
@@ -8,10 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gwen\Documents\GitHub\Factorio-Astra-Asteroids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB34B3ED-8EF0-4EE0-A22C-575C8BE4DE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773FF3E3-F152-4A0C-9E7D-050331793804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="4" xr2:uid="{19A80CD4-A61D-4139-863E-8E630E8C5493}"/>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="3" xr2:uid="{B83F7878-8263-4A97-A1DF-A9E638B23B4E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="4" xr2:uid="{B83F7878-8263-4A97-A1DF-A9E638B23B4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -75,7 +74,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="2">
+  <futureMetadata name="XLRICHVALUE" count="3">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -90,25 +89,35 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="2">
+  <valueMetadata count="3">
     <bk>
       <rc t="2" v="0"/>
     </bk>
     <bk>
       <rc t="2" v="1"/>
     </bk>
+    <bk>
+      <rc t="2" v="2"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="366">
   <si>
     <t>Metallic</t>
   </si>
@@ -14662,6 +14671,9 @@
   </si>
   <si>
     <t>"k[fulgora].z[special]"</t>
+  </si>
+  <si>
+    <t>string</t>
   </si>
 </sst>
 </file>
@@ -14838,7 +14850,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -14908,11 +14920,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="119">
+  <dxfs count="120">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -15070,10 +15093,6 @@
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -16222,23 +16241,23 @@
     <dataField name="Sum of EV" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="15">
-    <format dxfId="118">
+    <format dxfId="119">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="117">
+    <format dxfId="118">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="116">
+    <format dxfId="117">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="115">
+    <format dxfId="116">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="114">
+    <format dxfId="115">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="19">
@@ -16265,16 +16284,16 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="113">
+    <format dxfId="114">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="112">
+    <format dxfId="113">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="111">
+    <format dxfId="112">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="110">
+    <format dxfId="111">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="19">
@@ -16301,10 +16320,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="109">
+    <format dxfId="110">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="108">
+    <format dxfId="109">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="5">
@@ -16317,13 +16336,13 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="107">
+    <format dxfId="108">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="106">
+    <format dxfId="107">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="105">
+    <format dxfId="106">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="5">
@@ -16336,7 +16355,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="104">
+    <format dxfId="105">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -16427,7 +16446,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3">
   <rv s="0">
     <v>1</v>
     <v>8</v>
@@ -16438,11 +16457,15 @@
     <v>13</v>
     <v>3</v>
   </rv>
+  <rv s="2">
+    <v>13</v>
+    <v>1</v>
+  </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3">
   <s t="_error">
     <k n="colOffset" t="i"/>
     <k n="errorType" t="i"/>
@@ -16453,54 +16476,58 @@
     <k n="errorType" t="i"/>
     <k n="subType" t="i"/>
   </s>
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="propagated" t="b"/>
+  </s>
 </rvStructures>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9A0BFF85-5E25-44F5-989C-05E81AFBA27C}" name="Table4" displayName="Table4" ref="B3:AB25" totalsRowShown="0" headerRowDxfId="103">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9A0BFF85-5E25-44F5-989C-05E81AFBA27C}" name="Table4" displayName="Table4" ref="B3:AB25" totalsRowShown="0" headerRowDxfId="104">
   <autoFilter ref="B3:AB25" xr:uid="{9A0BFF85-5E25-44F5-989C-05E81AFBA27C}"/>
   <tableColumns count="27">
     <tableColumn id="1" xr3:uid="{B1A354A2-D591-4F7C-89E1-AB75527E5993}" name="Recipe"/>
-    <tableColumn id="27" xr3:uid="{1411294A-B7C7-4726-B55B-8DABEE6ED457}" name="energy_required" dataDxfId="102">
+    <tableColumn id="27" xr3:uid="{1411294A-B7C7-4726-B55B-8DABEE6ED457}" name="energy_required" dataDxfId="103">
       <calculatedColumnFormula>INDEX(Table7[energy_required], MATCH(Table4[[#This Row],[Recipe]], Table7[Recipe], 0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{7F80CA45-0C9C-4D9D-A37C-6DF3AD5E0BEB}" name="iron-ore" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{AC60A2AA-9D82-482D-A597-78045793B05D}" name="copper-ore" dataDxfId="100"/>
-    <tableColumn id="4" xr3:uid="{5029DD94-2977-4B99-94DB-19EA67D75D22}" name="carbon" dataDxfId="99"/>
-    <tableColumn id="5" xr3:uid="{52F010C3-27DB-43E9-A9D6-11A1C5DB092F}" name="sulfur" dataDxfId="98"/>
-    <tableColumn id="6" xr3:uid="{F06F185C-FC3F-465E-B9E4-758205B9F0F4}" name="ice" dataDxfId="97"/>
-    <tableColumn id="7" xr3:uid="{1554F3DE-DB8B-471F-922A-8D30297584F3}" name="calcite" dataDxfId="96"/>
-    <tableColumn id="8" xr3:uid="{E7F322CB-036A-403C-8BF8-6B20B8C6CCD1}" name="Oil Thing" dataDxfId="95">
+    <tableColumn id="2" xr3:uid="{7F80CA45-0C9C-4D9D-A37C-6DF3AD5E0BEB}" name="iron-ore" dataDxfId="102"/>
+    <tableColumn id="3" xr3:uid="{AC60A2AA-9D82-482D-A597-78045793B05D}" name="copper-ore" dataDxfId="101"/>
+    <tableColumn id="4" xr3:uid="{5029DD94-2977-4B99-94DB-19EA67D75D22}" name="carbon" dataDxfId="100"/>
+    <tableColumn id="5" xr3:uid="{52F010C3-27DB-43E9-A9D6-11A1C5DB092F}" name="sulfur" dataDxfId="99"/>
+    <tableColumn id="6" xr3:uid="{F06F185C-FC3F-465E-B9E4-758205B9F0F4}" name="ice" dataDxfId="98"/>
+    <tableColumn id="7" xr3:uid="{1554F3DE-DB8B-471F-922A-8D30297584F3}" name="calcite" dataDxfId="97"/>
+    <tableColumn id="8" xr3:uid="{E7F322CB-036A-403C-8BF8-6B20B8C6CCD1}" name="Oil Thing" dataDxfId="96">
       <calculatedColumnFormula array="1">_xlfn.LET(_xlpm.recipeResults, _xlfn._xlws.FILTER(Table7[[Results 1]:[Results 4]], Table7[Recipe] = Table4[[#This Row],[Recipe]]),
      IFERROR(
      _xlfn._xlws.FILTER(_xlpm.recipeResults, ISNUMBER(SEARCH(J$3, _xlpm.recipeResults))), " - ") )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="26" xr3:uid="{C4622E41-2D57-42C3-A31B-EF19C158ACB5}" name="solid-fuel" dataDxfId="94">
+    <tableColumn id="26" xr3:uid="{C4622E41-2D57-42C3-A31B-EF19C158ACB5}" name="solid-fuel" dataDxfId="95">
       <calculatedColumnFormula array="1">_xlfn.LET(_xlpm.recipeResults, _xlfn._xlws.FILTER(Table7[[Results 1]:[Results 4]], Table7[Recipe] = Table4[[#This Row],[Recipe]]),
      IFERROR(
      _xlfn._xlws.FILTER(_xlpm.recipeResults, ISNUMBER(SEARCH(K$3, _xlpm.recipeResults))), " - ") )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{F529E26B-0253-4C02-95D8-95DB987CD83E}" name="coal" dataDxfId="93"/>
-    <tableColumn id="10" xr3:uid="{D18F88A9-729A-4165-BA55-675D11D2231A}" name="stone" dataDxfId="92"/>
-    <tableColumn id="11" xr3:uid="{57DAEF24-F8A7-492C-9706-2674BFBB49E1}" name="uranium-ore" dataDxfId="91">
+    <tableColumn id="9" xr3:uid="{F529E26B-0253-4C02-95D8-95DB987CD83E}" name="coal" dataDxfId="94"/>
+    <tableColumn id="10" xr3:uid="{D18F88A9-729A-4165-BA55-675D11D2231A}" name="stone" dataDxfId="93"/>
+    <tableColumn id="11" xr3:uid="{57DAEF24-F8A7-492C-9706-2674BFBB49E1}" name="uranium-ore" dataDxfId="92">
       <calculatedColumnFormula array="1">_xlfn.LET(_xlpm.recipeResults, _xlfn._xlws.FILTER(Table7[[Results 1]:[Results 4]], Table7[Recipe] = Table4[[#This Row],[Recipe]]),
      IFERROR(
      _xlfn._xlws.FILTER(_xlpm.recipeResults, ISNUMBER(SEARCH(N$3, _xlpm.recipeResults))), " - ") )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{688FF19F-43DB-4F57-B5C7-CB20C171B5A5}" name="uranium-238" dataDxfId="90"/>
-    <tableColumn id="24" xr3:uid="{8B59E641-D762-475E-BE04-0AD557DA2633}" name="uranium-235" dataDxfId="89"/>
-    <tableColumn id="12" xr3:uid="{49325880-AB22-406C-9EBF-F9714278E54F}" name="tungsten-ore" dataDxfId="88"/>
-    <tableColumn id="25" xr3:uid="{4B574229-0587-4E11-816D-60F689340097}" name="lava" dataDxfId="87"/>
-    <tableColumn id="13" xr3:uid="{876F7B27-7476-478B-9F55-220BB73A33D4}" name="scrap" dataDxfId="86"/>
-    <tableColumn id="14" xr3:uid="{1D9F494D-4B80-42A5-85C3-6484CB3803F7}" name="yumako-seed" dataDxfId="85"/>
-    <tableColumn id="15" xr3:uid="{CC0EBC6A-4432-4CBA-A41B-E7B6031BD83F}" name="jellynut-seed" dataDxfId="84"/>
-    <tableColumn id="16" xr3:uid="{2B7FB235-2E10-4FA1-BC7C-964E7947466A}" name="spoilage" dataDxfId="83"/>
-    <tableColumn id="17" xr3:uid="{CEE0F52B-14B0-48FB-AD2F-A1A1A9DACF76}" name="Dormant Pentapod Egg" dataDxfId="82"/>
-    <tableColumn id="18" xr3:uid="{F34385CF-1935-4968-8261-48F21ADB2D44}" name="(tbd) ammonia" dataDxfId="81"/>
-    <tableColumn id="19" xr3:uid="{405DEB99-0752-4FA5-BCC3-09F744698489}" name="(tbd) flourine" dataDxfId="80"/>
-    <tableColumn id="20" xr3:uid="{ADD7E20E-3FB5-4185-8AD9-7781DF09236F}" name="(tbd) lithium" dataDxfId="79"/>
-    <tableColumn id="21" xr3:uid="{82818854-DC1B-485E-9809-F8B0261BEDE0}" name="(tbd) promethium" dataDxfId="78"/>
-    <tableColumn id="22" xr3:uid="{5634330F-FEBB-4799-90EC-922642138192}" name="Holmium Solution" dataDxfId="77"/>
+    <tableColumn id="23" xr3:uid="{688FF19F-43DB-4F57-B5C7-CB20C171B5A5}" name="uranium-238" dataDxfId="91"/>
+    <tableColumn id="24" xr3:uid="{8B59E641-D762-475E-BE04-0AD557DA2633}" name="uranium-235" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{49325880-AB22-406C-9EBF-F9714278E54F}" name="tungsten-ore" dataDxfId="89"/>
+    <tableColumn id="25" xr3:uid="{4B574229-0587-4E11-816D-60F689340097}" name="lava" dataDxfId="88"/>
+    <tableColumn id="13" xr3:uid="{876F7B27-7476-478B-9F55-220BB73A33D4}" name="scrap" dataDxfId="87"/>
+    <tableColumn id="14" xr3:uid="{1D9F494D-4B80-42A5-85C3-6484CB3803F7}" name="yumako-seed" dataDxfId="86"/>
+    <tableColumn id="15" xr3:uid="{CC0EBC6A-4432-4CBA-A41B-E7B6031BD83F}" name="jellynut-seed" dataDxfId="85"/>
+    <tableColumn id="16" xr3:uid="{2B7FB235-2E10-4FA1-BC7C-964E7947466A}" name="spoilage" dataDxfId="84"/>
+    <tableColumn id="17" xr3:uid="{CEE0F52B-14B0-48FB-AD2F-A1A1A9DACF76}" name="Dormant Pentapod Egg" dataDxfId="83"/>
+    <tableColumn id="18" xr3:uid="{F34385CF-1935-4968-8261-48F21ADB2D44}" name="(tbd) ammonia" dataDxfId="82"/>
+    <tableColumn id="19" xr3:uid="{405DEB99-0752-4FA5-BCC3-09F744698489}" name="(tbd) flourine" dataDxfId="81"/>
+    <tableColumn id="20" xr3:uid="{ADD7E20E-3FB5-4185-8AD9-7781DF09236F}" name="(tbd) lithium" dataDxfId="80"/>
+    <tableColumn id="21" xr3:uid="{82818854-DC1B-485E-9809-F8B0261BEDE0}" name="(tbd) promethium" dataDxfId="79"/>
+    <tableColumn id="22" xr3:uid="{5634330F-FEBB-4799-90EC-922642138192}" name="Holmium Solution" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -16515,18 +16542,18 @@
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{EFD8865D-C9ED-4BA8-B73C-113EDAD68DA5}" name="Variable's Name"/>
     <tableColumn id="3" xr3:uid="{1A67492A-77CF-48AB-9609-594DA5CCF328}" name="name"/>
-    <tableColumn id="2" xr3:uid="{587148E6-4B98-4DD4-8691-6E43006C9E89}" name="type" dataDxfId="76">
+    <tableColumn id="2" xr3:uid="{587148E6-4B98-4DD4-8691-6E43006C9E89}" name="type" dataDxfId="77">
       <calculatedColumnFormula>"""item"""</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{4C2D2AEB-4928-4F13-91B0-2184B98F54BD}" name="subgroup" dataDxfId="75">
+    <tableColumn id="4" xr3:uid="{4C2D2AEB-4928-4F13-91B0-2184B98F54BD}" name="subgroup" dataDxfId="76">
       <calculatedColumnFormula>"""space-material"""</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{A45CDEC7-39DE-4333-8E31-011D04DA2762}" name="order"/>
     <tableColumn id="6" xr3:uid="{499C643B-C1ED-4A32-BE42-9946CC52BC6E}" name="icon"/>
-    <tableColumn id="7" xr3:uid="{834AC55A-1278-424D-94B7-2EDF700340B6}" name="stack_size" dataDxfId="74">
+    <tableColumn id="7" xr3:uid="{834AC55A-1278-424D-94B7-2EDF700340B6}" name="stack_size" dataDxfId="75">
       <calculatedColumnFormula>1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{9145470B-0772-4705-8B45-24698F613F56}" name="full string" dataDxfId="73">
+    <tableColumn id="8" xr3:uid="{9145470B-0772-4705-8B45-24698F613F56}" name="full string" dataDxfId="74">
       <calculatedColumnFormula array="1">_xlfn.TEXTJOIN("
 ", TRUE, Chunk_Items[[#This Row],[Variable''s Name]] &amp; "." &amp; Chunk_Items[[#Headers],[name]:[stack_size]] &amp; " = " &amp; Chunk_Items[[#This Row],[name]:[stack_size]])</calculatedColumnFormula>
     </tableColumn>
@@ -16544,13 +16571,13 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{9C8B2B85-651A-48F5-BE74-6B0CB5EC6401}" name="Variable's Name"/>
     <tableColumn id="3" xr3:uid="{5CB5E631-FE01-4CDD-A4B3-008A4C86A223}" name="name"/>
-    <tableColumn id="2" xr3:uid="{36E1B303-2D0B-4894-BA0E-22315D6AA6E7}" name="type" dataDxfId="72">
+    <tableColumn id="2" xr3:uid="{36E1B303-2D0B-4894-BA0E-22315D6AA6E7}" name="type" dataDxfId="73">
       <calculatedColumnFormula>"""asteroid-chunk"""</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{33E8079D-0ADE-49CC-8F5F-FB561D1043C6}" name="minable" dataDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{33E8079D-0ADE-49CC-8F5F-FB561D1043C6}" name="minable" dataDxfId="72"/>
     <tableColumn id="5" xr3:uid="{2D398BB0-41AE-40CE-AA0F-6FA6647FFA57}" name="order"/>
     <tableColumn id="6" xr3:uid="{82F86FA9-1FFF-4AFF-A528-DD559BDA3930}" name="icon"/>
-    <tableColumn id="7" xr3:uid="{8D2BAF1D-A998-4CFE-AE20-A7C5A809314F}" name="full string" dataDxfId="70">
+    <tableColumn id="7" xr3:uid="{8D2BAF1D-A998-4CFE-AE20-A7C5A809314F}" name="full string" dataDxfId="71">
       <calculatedColumnFormula array="1">_xlfn.TEXTJOIN("
 ", TRUE, Chunks[[#This Row],[Variable''s Name]] &amp; "." &amp; Chunks[[#Headers],[name]:[icon]] &amp; " = " &amp; Chunks[[#This Row],[name]:[icon]])</calculatedColumnFormula>
     </tableColumn>
@@ -16563,28 +16590,28 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E53CB6FB-2E2C-443B-95B1-3E2AFFD034E2}" name="Table7_1" displayName="Table7_1" ref="A1:Y21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:Y21" xr:uid="{E53CB6FB-2E2C-443B-95B1-3E2AFFD034E2}"/>
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{25B70940-94F8-4DB8-88CD-A28BB25BF46D}" uniqueName="1" name="Recipe" queryTableFieldId="1" dataDxfId="69"/>
-    <tableColumn id="2" xr3:uid="{6938BA52-64B5-4541-85FE-0568CF57BE53}" uniqueName="2" name="Unwritten?" queryTableFieldId="2" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{25B70940-94F8-4DB8-88CD-A28BB25BF46D}" uniqueName="1" name="Recipe" queryTableFieldId="1" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{6938BA52-64B5-4541-85FE-0568CF57BE53}" uniqueName="2" name="Unwritten?" queryTableFieldId="2" dataDxfId="69"/>
     <tableColumn id="3" xr3:uid="{1B648304-5C74-4610-8A43-DF788A2F0682}" uniqueName="3" name="Advanced?" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{71899E0C-12BA-4960-936B-611EB515C0AC}" uniqueName="4" name="Variable's Name" queryTableFieldId="4" dataDxfId="67"/>
-    <tableColumn id="5" xr3:uid="{47AADCB0-91CC-4ACD-BC22-48C0ABAD5DDF}" uniqueName="5" name="name" queryTableFieldId="5" dataDxfId="66"/>
-    <tableColumn id="6" xr3:uid="{0AAE9926-1717-4A7C-81EF-968AF648698F}" uniqueName="6" name="Result_1_type" queryTableFieldId="6" dataDxfId="65"/>
-    <tableColumn id="7" xr3:uid="{B8E38A26-43C7-4117-B451-06DBBE98CF09}" uniqueName="7" name="Result_1_name" queryTableFieldId="7" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{71899E0C-12BA-4960-936B-611EB515C0AC}" uniqueName="4" name="Variable's Name" queryTableFieldId="4" dataDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{47AADCB0-91CC-4ACD-BC22-48C0ABAD5DDF}" uniqueName="5" name="name" queryTableFieldId="5" dataDxfId="67"/>
+    <tableColumn id="6" xr3:uid="{0AAE9926-1717-4A7C-81EF-968AF648698F}" uniqueName="6" name="Result_1_type" queryTableFieldId="6" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{B8E38A26-43C7-4117-B451-06DBBE98CF09}" uniqueName="7" name="Result_1_name" queryTableFieldId="7" dataDxfId="65"/>
     <tableColumn id="8" xr3:uid="{232E0949-6EC0-4070-B3B6-D5527152EC92}" uniqueName="8" name="Result_1_amt_min" queryTableFieldId="8"/>
     <tableColumn id="9" xr3:uid="{406E71DF-32D1-4345-A52D-B7D3102D97F3}" uniqueName="9" name="Result_1_amt_max" queryTableFieldId="9"/>
     <tableColumn id="10" xr3:uid="{D6695C50-86D7-422B-926F-5110F80F5466}" uniqueName="10" name="Result_1_P" queryTableFieldId="10"/>
-    <tableColumn id="11" xr3:uid="{12F89D76-7449-448D-98CC-D411D1475A3E}" uniqueName="11" name="Result_2_type" queryTableFieldId="11" dataDxfId="63"/>
-    <tableColumn id="12" xr3:uid="{586F2CF2-DA91-4E08-AD5D-AE1B76BC7EC0}" uniqueName="12" name="Result_2_name" queryTableFieldId="12" dataDxfId="62"/>
+    <tableColumn id="11" xr3:uid="{12F89D76-7449-448D-98CC-D411D1475A3E}" uniqueName="11" name="Result_2_type" queryTableFieldId="11" dataDxfId="64"/>
+    <tableColumn id="12" xr3:uid="{586F2CF2-DA91-4E08-AD5D-AE1B76BC7EC0}" uniqueName="12" name="Result_2_name" queryTableFieldId="12" dataDxfId="63"/>
     <tableColumn id="13" xr3:uid="{591FD322-8C8B-4CEA-ADEC-225C7718C7EA}" uniqueName="13" name="Result_2_amt_min" queryTableFieldId="13"/>
     <tableColumn id="14" xr3:uid="{35B09536-BD39-4556-A5A6-8B26833986F8}" uniqueName="14" name="Result_2_amt_max" queryTableFieldId="14"/>
     <tableColumn id="15" xr3:uid="{D7B93839-634E-4DAC-A31C-74371349085E}" uniqueName="15" name="Result_2_P" queryTableFieldId="15"/>
-    <tableColumn id="16" xr3:uid="{173610F8-5BDC-4DC9-8017-BD40CD5A84C2}" uniqueName="16" name="Result_3_type" queryTableFieldId="16" dataDxfId="61"/>
-    <tableColumn id="17" xr3:uid="{A26C6901-F141-49CF-93BE-A3486152942F}" uniqueName="17" name="Result_3_name" queryTableFieldId="17" dataDxfId="60"/>
+    <tableColumn id="16" xr3:uid="{173610F8-5BDC-4DC9-8017-BD40CD5A84C2}" uniqueName="16" name="Result_3_type" queryTableFieldId="16" dataDxfId="62"/>
+    <tableColumn id="17" xr3:uid="{A26C6901-F141-49CF-93BE-A3486152942F}" uniqueName="17" name="Result_3_name" queryTableFieldId="17" dataDxfId="61"/>
     <tableColumn id="18" xr3:uid="{9D777C1E-B7F3-4D13-9252-6FA1242AC1C6}" uniqueName="18" name="Result_3_amt_min" queryTableFieldId="18"/>
     <tableColumn id="19" xr3:uid="{B85EEF5E-B938-4781-8FDD-89BA612694AB}" uniqueName="19" name="Result_3_amt_max" queryTableFieldId="19"/>
     <tableColumn id="20" xr3:uid="{CF44E894-9365-4B08-A015-D19576C0C054}" uniqueName="20" name="Result_3_P" queryTableFieldId="20"/>
-    <tableColumn id="21" xr3:uid="{4191E007-5B61-405E-834E-CB82EC4E6D01}" uniqueName="21" name="Result_4_type" queryTableFieldId="21" dataDxfId="59"/>
-    <tableColumn id="22" xr3:uid="{6E00A2BA-308B-4E79-AE13-BA2B7FF3266E}" uniqueName="22" name="Result_4_name" queryTableFieldId="22" dataDxfId="58"/>
+    <tableColumn id="21" xr3:uid="{4191E007-5B61-405E-834E-CB82EC4E6D01}" uniqueName="21" name="Result_4_type" queryTableFieldId="21" dataDxfId="60"/>
+    <tableColumn id="22" xr3:uid="{6E00A2BA-308B-4E79-AE13-BA2B7FF3266E}" uniqueName="22" name="Result_4_name" queryTableFieldId="22" dataDxfId="59"/>
     <tableColumn id="23" xr3:uid="{B08DA47E-615C-42A2-B48F-E089661FB480}" uniqueName="23" name="Result_4_amt_min" queryTableFieldId="23"/>
     <tableColumn id="24" xr3:uid="{80FE8B91-761C-4A2E-84E2-899EEE89286A}" uniqueName="24" name="Result_4_amt_max" queryTableFieldId="24"/>
     <tableColumn id="25" xr3:uid="{B57634A6-34CE-4EA5-9B05-C8F84F58A41A}" uniqueName="25" name="Result_4_P" queryTableFieldId="25"/>
@@ -16594,126 +16621,126 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{996E5AF8-4762-451C-9EC5-44266BFF352B}" name="Table7" displayName="Table7" ref="C7:AP28" totalsRowShown="0" headerRowDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{996E5AF8-4762-451C-9EC5-44266BFF352B}" name="Table7" displayName="Table7" ref="C7:AP28" totalsRowShown="0" headerRowDxfId="58">
   <autoFilter ref="C7:AP28" xr:uid="{996E5AF8-4762-451C-9EC5-44266BFF352B}"/>
   <tableColumns count="40">
     <tableColumn id="1" xr3:uid="{1C7B22C3-8503-40CA-B985-0F11F98EB3C6}" name="Recipe"/>
-    <tableColumn id="12" xr3:uid="{44C30B7E-3F48-43EE-A476-EAF4BA20C75A}" name="Unwritten?" dataDxfId="56"/>
-    <tableColumn id="41" xr3:uid="{6E5608DA-75C3-48D4-92AF-824B8C6B9141}" name="Advanced?" dataDxfId="55">
+    <tableColumn id="12" xr3:uid="{44C30B7E-3F48-43EE-A476-EAF4BA20C75A}" name="Unwritten?" dataDxfId="57"/>
+    <tableColumn id="41" xr3:uid="{6E5608DA-75C3-48D4-92AF-824B8C6B9141}" name="Advanced?" dataDxfId="56">
       <calculatedColumnFormula>OR(ISNUMBER(SEARCH("Adv", Table7[[#This Row],[Recipe]])), ISNUMBER(SEARCH("Special", Table7[[#This Row],[Recipe]])))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{D73BFE2A-2B7F-460C-B8F4-2293AE8F1CDF}" name="Variable's Name" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{E995243B-09A0-4B61-9891-2750A2869DC3}" name="name" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{503397F1-8755-4CF0-8F78-A9F7740B5790}" name="icon" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{68F82173-B464-4B40-AC23-3E4F9BE9F52A}" name="order" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{41FF6C48-F0D3-46AF-A21F-51ACC01FAB0C}" name="enabled" dataDxfId="50"/>
-    <tableColumn id="14" xr3:uid="{D9A98507-2FB7-4229-B1C0-4B1DA8557E9F}" name="energy_required" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{49007205-346D-4C29-AD68-C79FA0EA720B}" name="Ingredient 1" dataDxfId="48"/>
-    <tableColumn id="15" xr3:uid="{805B845F-9765-4945-826D-8F506E139BE2}" name="Ingredient 2" dataDxfId="47"/>
-    <tableColumn id="16" xr3:uid="{D892DCC1-CA40-40C6-A026-DE02CB8B8541}" name="Ingredient 1 Amount" dataDxfId="46"/>
-    <tableColumn id="17" xr3:uid="{043F0671-10F0-435E-93F6-76D671AC8761}" name="Ingredient 2 Amount" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{8EF822E8-07FB-4876-8800-25F2A9B81873}" name="Result_1_type" dataDxfId="0">
+    <tableColumn id="39" xr3:uid="{D73BFE2A-2B7F-460C-B8F4-2293AE8F1CDF}" name="Variable's Name" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{E995243B-09A0-4B61-9891-2750A2869DC3}" name="name" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{503397F1-8755-4CF0-8F78-A9F7740B5790}" name="icon" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{68F82173-B464-4B40-AC23-3E4F9BE9F52A}" name="order" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{41FF6C48-F0D3-46AF-A21F-51ACC01FAB0C}" name="enabled" dataDxfId="51"/>
+    <tableColumn id="14" xr3:uid="{D9A98507-2FB7-4229-B1C0-4B1DA8557E9F}" name="energy_required" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{49007205-346D-4C29-AD68-C79FA0EA720B}" name="Ingredient 1" dataDxfId="49"/>
+    <tableColumn id="15" xr3:uid="{805B845F-9765-4945-826D-8F506E139BE2}" name="Ingredient 2" dataDxfId="48"/>
+    <tableColumn id="16" xr3:uid="{D892DCC1-CA40-40C6-A026-DE02CB8B8541}" name="Ingredient 1 Amount" dataDxfId="47"/>
+    <tableColumn id="17" xr3:uid="{043F0671-10F0-435E-93F6-76D671AC8761}" name="Ingredient 2 Amount" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{8EF822E8-07FB-4876-8800-25F2A9B81873}" name="Result_1_type" dataDxfId="2">
       <calculatedColumnFormula array="1">INDEX(Table8[type], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="30" xr3:uid="{36B4E4F7-052E-4455-A6CA-FFCC3E9245F7}" name="Result_1_name" dataDxfId="20">
+    <tableColumn id="30" xr3:uid="{36B4E4F7-052E-4455-A6CA-FFCC3E9245F7}" name="Result_1_name" dataDxfId="22">
       <calculatedColumnFormula array="1">INDEX(Table8[name], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{9C3D4CEF-5F40-4B68-BD87-448388551748}" name="Result_1_amt_min" dataDxfId="19">
+    <tableColumn id="27" xr3:uid="{9C3D4CEF-5F40-4B68-BD87-448388551748}" name="Result_1_amt_min" dataDxfId="21">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_min], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="26" xr3:uid="{F871C881-69CD-4795-AB43-8B752D2E5250}" name="Result_1_amt_max" dataDxfId="18">
+    <tableColumn id="26" xr3:uid="{F871C881-69CD-4795-AB43-8B752D2E5250}" name="Result_1_amt_max" dataDxfId="20">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_max], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{6E355266-0C10-4989-9F5C-656E5531B809}" name="Result_1_P" dataDxfId="17">
+    <tableColumn id="28" xr3:uid="{6E355266-0C10-4989-9F5C-656E5531B809}" name="Result_1_P" dataDxfId="19">
       <calculatedColumnFormula array="1">INDEX(Table8[P], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{F666EFD4-EFAB-4ED2-9F8C-93F381615487}" name="Result_2_type" dataDxfId="15">
+    <tableColumn id="34" xr3:uid="{F666EFD4-EFAB-4ED2-9F8C-93F381615487}" name="Result_2_type" dataDxfId="17">
       <calculatedColumnFormula array="1">INDEX(Table8[type], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="31" xr3:uid="{EBAA7D64-5ABB-4E65-8B5B-00682D717ECF}" name="Result_2_name" dataDxfId="14">
+    <tableColumn id="31" xr3:uid="{EBAA7D64-5ABB-4E65-8B5B-00682D717ECF}" name="Result_2_name" dataDxfId="16">
       <calculatedColumnFormula array="1">INDEX(Table8[name], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{0F604324-0BE1-40EA-BC68-971D78B203CD}" name="Result_2_amt_min" dataDxfId="13">
+    <tableColumn id="22" xr3:uid="{0F604324-0BE1-40EA-BC68-971D78B203CD}" name="Result_2_amt_min" dataDxfId="15">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_min], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{95845240-17DF-4258-A672-6BC4AC4F0623}" name="Result_2_amt_max" dataDxfId="12">
+    <tableColumn id="29" xr3:uid="{95845240-17DF-4258-A672-6BC4AC4F0623}" name="Result_2_amt_max" dataDxfId="14">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_max], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{F05C630D-F7F6-4014-91DB-C5753DF18CBC}" name="Result_2_P" dataDxfId="11">
+    <tableColumn id="23" xr3:uid="{F05C630D-F7F6-4014-91DB-C5753DF18CBC}" name="Result_2_P" dataDxfId="13">
       <calculatedColumnFormula array="1">INDEX(Table8[P], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="35" xr3:uid="{29FDA9C5-AC15-474C-B065-A8F35BA59418}" name="Result_3_type" dataDxfId="10">
+    <tableColumn id="35" xr3:uid="{29FDA9C5-AC15-474C-B065-A8F35BA59418}" name="Result_3_type" dataDxfId="12">
       <calculatedColumnFormula array="1">INDEX(Table8[type], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="32" xr3:uid="{9317562F-B7E9-490E-BFBC-0F03122AB5F9}" name="Result_3_name" dataDxfId="9">
+    <tableColumn id="32" xr3:uid="{9317562F-B7E9-490E-BFBC-0F03122AB5F9}" name="Result_3_name" dataDxfId="11">
       <calculatedColumnFormula array="1">INDEX(Table8[name], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="25" xr3:uid="{04B02B68-0016-44BE-8B0D-6E6053EB4293}" name="Result_3_amt_min" dataDxfId="8">
+    <tableColumn id="25" xr3:uid="{04B02B68-0016-44BE-8B0D-6E6053EB4293}" name="Result_3_amt_min" dataDxfId="10">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_min], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{4A76DB66-F126-4A19-B7B9-052150F5EC16}" name="Result_3_amt_max" dataDxfId="7">
+    <tableColumn id="24" xr3:uid="{4A76DB66-F126-4A19-B7B9-052150F5EC16}" name="Result_3_amt_max" dataDxfId="9">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_max], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{1834E88C-3996-4B83-A2D6-E4CBF6799983}" name="Result_3_P" dataDxfId="6">
+    <tableColumn id="18" xr3:uid="{1834E88C-3996-4B83-A2D6-E4CBF6799983}" name="Result_3_P" dataDxfId="8">
       <calculatedColumnFormula array="1">INDEX(Table8[P], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="36" xr3:uid="{5C2D1484-E711-4E82-92DB-57B04BD66315}" name="Result_4_type" dataDxfId="5">
+    <tableColumn id="36" xr3:uid="{5C2D1484-E711-4E82-92DB-57B04BD66315}" name="Result_4_type" dataDxfId="7">
       <calculatedColumnFormula array="1">INDEX(Table8[type], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="33" xr3:uid="{5A6880AC-0CDF-4FF5-95A6-EF019821685D}" name="Result_4_name" dataDxfId="4">
+    <tableColumn id="33" xr3:uid="{5A6880AC-0CDF-4FF5-95A6-EF019821685D}" name="Result_4_name" dataDxfId="6">
       <calculatedColumnFormula array="1">INDEX(Table8[name], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{F27B8545-BFA0-4FA2-BC1B-A026F34E43F0}" name="Result_4_amt_min" dataDxfId="3">
+    <tableColumn id="20" xr3:uid="{F27B8545-BFA0-4FA2-BC1B-A026F34E43F0}" name="Result_4_amt_min" dataDxfId="5">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_min], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{A869DC81-85C7-4615-8A5E-CD93FEADF931}" name="Result_4_amt_max" dataDxfId="2">
+    <tableColumn id="19" xr3:uid="{A869DC81-85C7-4615-8A5E-CD93FEADF931}" name="Result_4_amt_max" dataDxfId="4">
       <calculatedColumnFormula array="1">INDEX(Table8[amount_max], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{C5FEE21E-C6E2-49F8-AD36-B9EED8A7B149}" name="Result_4_P" dataDxfId="1">
+    <tableColumn id="21" xr3:uid="{C5FEE21E-C6E2-49F8-AD36-B9EED8A7B149}" name="Result_4_P" dataDxfId="3">
       <calculatedColumnFormula array="1">INDEX(Table8[P], MATCH(Table7[[#This Row],[Recipe]], Table8[Recipe], 0) + 3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{33C291CA-AEA3-41A6-8665-03327AB3E806}" name="Results 1" dataDxfId="44">
+    <tableColumn id="8" xr3:uid="{33C291CA-AEA3-41A6-8665-03327AB3E806}" name="Results 1" dataDxfId="45">
       <calculatedColumnFormula array="1">IF(ISBLANK(Table7[[#This Row],[Result_1_type]]), FALSE, "{ " &amp;
  _xlfn.TEXTJOIN(", ",
           TRUE,
           {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table7[[#This Row],[Result_1_type]:[Result_1_P]])), """" &amp; Table7[[#This Row],[Result_1_type]:[Result_1_P]] &amp; """", Table7[[#This Row],[Result_1_type]:[Result_1_P]]) ) &amp;
   " }" )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{7BF645B9-19D0-4473-ACE6-12B66A8165AE}" name="Results 2" dataDxfId="43">
+    <tableColumn id="9" xr3:uid="{7BF645B9-19D0-4473-ACE6-12B66A8165AE}" name="Results 2" dataDxfId="44">
       <calculatedColumnFormula array="1">IF(ISBLANK(Table7[[#This Row],[Result_2_type]]), FALSE, "{ " &amp;
  _xlfn.TEXTJOIN(", ",
           TRUE,
           {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table7[[#This Row],[Result_2_type]:[Result_2_P]])), """" &amp; Table7[[#This Row],[Result_2_type]:[Result_2_P]] &amp; """", Table7[[#This Row],[Result_2_type]:[Result_2_P]]) ) &amp;
   " }" )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{73804FC8-69EB-4E05-8650-4BB574DE531D}" name="Results 3" dataDxfId="42">
+    <tableColumn id="10" xr3:uid="{73804FC8-69EB-4E05-8650-4BB574DE531D}" name="Results 3" dataDxfId="43">
       <calculatedColumnFormula array="1">IF(ISBLANK(Table7[[#This Row],[Result_3_type]]), FALSE, "{ " &amp;
  _xlfn.TEXTJOIN(", ",
           TRUE,
           {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table7[[#This Row],[Result_3_type]:[Result_3_P]])), """" &amp; Table7[[#This Row],[Result_3_type]:[Result_3_P]] &amp; """", Table7[[#This Row],[Result_3_type]:[Result_3_P]]) ) &amp;
   " }" )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{6B40EA3E-9F3D-4135-BC18-3EC5AE95AEF0}" name="Results 4" dataDxfId="41">
+    <tableColumn id="11" xr3:uid="{6B40EA3E-9F3D-4135-BC18-3EC5AE95AEF0}" name="Results 4" dataDxfId="42">
       <calculatedColumnFormula array="1">IF(ISBLANK(Table7[[#This Row],[Result_4_type]]), FALSE, "{ " &amp;
  _xlfn.TEXTJOIN(", ",
           TRUE,
           {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table7[[#This Row],[Result_4_type]:[Result_4_P]])), """" &amp; Table7[[#This Row],[Result_4_type]:[Result_4_P]] &amp; """", Table7[[#This Row],[Result_4_type]:[Result_4_P]]) ) &amp;
   " }" )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{983E9E0D-A8BE-4A49-88C0-0F9647C154FB}" name="Ingredient String" dataDxfId="40">
+    <tableColumn id="13" xr3:uid="{983E9E0D-A8BE-4A49-88C0-0F9647C154FB}" name="Ingredient String" dataDxfId="41">
       <calculatedColumnFormula array="1" xml:space="preserve"> "{ " &amp;
  _xlfn.TEXTJOIN(", ",
           TRUE,
           "{ type = ""item"", name = """ &amp; _xlfn.TRIMRANGE(Table7[[#This Row],[Ingredient 1]:[Ingredient 2]]) &amp; """, amount = " &amp; _xlfn.TRIMRANGE(Table7[[#This Row],[Ingredient 1 Amount]:[Ingredient 2 Amount]]) &amp; " }")
 &amp; " }"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="37" xr3:uid="{D9725653-650B-4E33-86E4-FA48D30F5455}" name="Results String" dataDxfId="39">
+    <tableColumn id="37" xr3:uid="{D9725653-650B-4E33-86E4-FA48D30F5455}" name="Results String" dataDxfId="0">
       <calculatedColumnFormula array="1" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="40" xr3:uid="{6A447D5A-EAF2-404F-A826-F6177D7B50D6}" name="Whole String" dataDxfId="38">
+    <tableColumn id="40" xr3:uid="{6A447D5A-EAF2-404F-A826-F6177D7B50D6}" name="Whole String" dataDxfId="40">
       <calculatedColumnFormula array="1">_xlfn.TEXTJOIN("
 ", TRUE, Table7[[#This Row],[Variable''s Name]] &amp; "." &amp; Table7[[#Headers],[name]:[energy_required]] &amp; " = " &amp; Table7[[#This Row],[name]:[energy_required]]) &amp; "
 " &amp; Table7[[#This Row],[Variable''s Name]] &amp; ".ingredients = " &amp; Table7[[#This Row],[Ingredient String]] &amp; "
@@ -16725,29 +16752,36 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EA71830A-828F-4695-B2FD-24C049275861}" name="Table8" displayName="Table8" ref="B3:K59" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
-  <autoFilter ref="B3:K59" xr:uid="{EA71830A-828F-4695-B2FD-24C049275861}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EA71830A-828F-4695-B2FD-24C049275861}" name="Table8" displayName="Table8" ref="B3:L59" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+  <autoFilter ref="B3:L59" xr:uid="{EA71830A-828F-4695-B2FD-24C049275861}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:K59">
     <sortCondition descending="1" ref="B3:B59"/>
   </sortState>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{125DA46D-9742-4063-80AF-7B3BD16A90B4}" name="Recipe" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{FB3F6848-8BA0-4CF9-94C5-347F36A39CF0}" name="type" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{2F1240D4-2D99-4EA6-9B56-7EE74D6AFB8B}" name="name" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{3BB9F2BA-0C22-4457-A366-03C34CF2C7C7}" name="amount_min" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{3D12B4DB-2238-43D9-B668-BBD3ED397240}" name="amount_max" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{218ABFBF-C1D6-4C94-A67C-3C2D682E3A95}" name="P" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{5E531594-85F5-4CD1-B27E-BC7800E08050}" name="Duration" dataDxfId="29">
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{125DA46D-9742-4063-80AF-7B3BD16A90B4}" name="Recipe" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{FB3F6848-8BA0-4CF9-94C5-347F36A39CF0}" name="type" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{2F1240D4-2D99-4EA6-9B56-7EE74D6AFB8B}" name="name" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{3BB9F2BA-0C22-4457-A366-03C34CF2C7C7}" name="amount_min" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{3D12B4DB-2238-43D9-B668-BBD3ED397240}" name="amount_max" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{218ABFBF-C1D6-4C94-A67C-3C2D682E3A95}" name="P" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{5E531594-85F5-4CD1-B27E-BC7800E08050}" name="Duration" dataDxfId="31">
       <calculatedColumnFormula>INDEX(Table7[energy_required], MATCH(Table8[[#This Row],[Recipe]], Table7[Recipe], 0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3EF6D105-597F-4C54-B302-4F46B4BD461A}" name="EV" dataDxfId="28">
+    <tableColumn id="7" xr3:uid="{3EF6D105-597F-4C54-B302-4F46B4BD461A}" name="EV" dataDxfId="30">
       <calculatedColumnFormula>AVERAGE(Table8[[#This Row],[amount_min]], Table8[[#This Row],[amount_max]]) * Table8[[#This Row],[P]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{0DE8515B-F44B-493D-B0E5-618AD508AA55}" name="EV/s" dataDxfId="27">
+    <tableColumn id="9" xr3:uid="{0DE8515B-F44B-493D-B0E5-618AD508AA55}" name="EV/s" dataDxfId="29">
       <calculatedColumnFormula>Table8[[#This Row],[EV]] / Table8[[#This Row],[Duration]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{2B62D157-F7A9-40B5-828B-0C9C0816CD17}" name="s/EV" dataDxfId="26">
+    <tableColumn id="10" xr3:uid="{2B62D157-F7A9-40B5-828B-0C9C0816CD17}" name="s/EV" dataDxfId="28">
       <calculatedColumnFormula>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{4856F71F-096D-4C64-84BD-AB3EF681F7DF}" name="string" dataDxfId="1">
+      <calculatedColumnFormula array="1">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -16759,11 +16793,11 @@
   <autoFilter ref="H5:K15" xr:uid="{8FC02366-D4DD-41A4-8050-773DDA42B27E}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{959EF51D-F84A-47B3-BB90-19C907903580}" name="name"/>
-    <tableColumn id="2" xr3:uid="{C3C91221-23BC-4002-9309-7C9CD86A66DB}" name="type" dataDxfId="25">
+    <tableColumn id="2" xr3:uid="{C3C91221-23BC-4002-9309-7C9CD86A66DB}" name="type" dataDxfId="27">
       <calculatedColumnFormula>"""item"""</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{214E8F8E-48B4-4BB8-B3A1-54F2A217D484}" name="amount"/>
-    <tableColumn id="7" xr3:uid="{24D768D4-2DBF-4BCF-BF27-3E53FCF0468E}" name="line items" dataDxfId="24">
+    <tableColumn id="7" xr3:uid="{24D768D4-2DBF-4BCF-BF27-3E53FCF0468E}" name="line items" dataDxfId="26">
       <calculatedColumnFormula array="1">"    { " &amp; _xlfn.TEXTJOIN(", ", TRUE, Table1[[#Headers],[name]:[amount]] &amp; " = " &amp; Table1[[#This Row],[name]:[amount]]) &amp; " }"</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -18687,7 +18721,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="B17:AB17">
-    <cfRule type="expression" dxfId="23" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="25" priority="1" stopIfTrue="1">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20367,9 +20401,6 @@
 local gleba_asteroid_chunk_crushing = table.deepcopy(data.raw.recipe["metallic-asteroid-crushing"])
 local fulgoran_asteroid_chunk_crushing = table.deepcopy(data.raw.recipe["metallic-asteroid-crushing"])
 local aquilo-asteroid-chunk_crushing = table.deepcopy(data.raw.recipe["metallic-asteroid-crushing"])
-local  = table.deepcopy(data.raw.recipe["advanced-metallic-asteroid-crushing"])
-local  = table.deepcopy(data.raw.recipe["advanced-metallic-asteroid-crushing"])
-local  = table.deepcopy(data.raw.recipe["advanced-metallic-asteroid-crushing"])
 local vulcanis_asteroid_chunk_crushing_adv = table.deepcopy(data.raw.recipe["advanced-metallic-asteroid-crushing"])
 local nauvis_asteroid_chunk_crushing_adv = table.deepcopy(data.raw.recipe["advanced-metallic-asteroid-crushing"])
 local gleba_asteroid_chunk_crushing_adv = table.deepcopy(data.raw.recipe["advanced-metallic-asteroid-crushing"])
@@ -20388,10 +20419,156 @@
       <c r="B4" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="12" t="e" cm="1">
+      <c r="C4" s="12" t="str" cm="1">
         <f t="array" ref="C4">_xlfn.TEXTJOIN("
 ", TRUE, _xlfn._xlws.FILTER(Table7[Whole String], ISBLANK(Table7[Unwritten?])))</f>
-        <v>#REF!</v>
+        <v>crude_asteroid_chunk_crushing.name = "astra-crude-asteroid-crushing"
+crude_asteroid_chunk_crushing.icon = "__Astra-Asteroids__/graphics/crude_crushing_basic.png"
+crude_asteroid_chunk_crushing.order = "g[crude].a[basic]"
+crude_asteroid_chunk_crushing.enabled = false
+crude_asteroid_chunk_crushing.energy_required = 2
+crude_asteroid_chunk_crushing.ingredients = { { type = "item", name = "astra-crude-asteroid-chunk", amount = 1 } }
+crude_asteroid_chunk_crushing.results = { 
+    { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
+    { type = "item", name = "astra-oilstone", amount_min = 4, amount_max = 5, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+}
+vulcanus_asteroid_chunk_crushing.name = "astra-vulcanus-asteroid-crushing"
+vulcanus_asteroid_chunk_crushing.icon = "__Astra-Asteroids__/graphics/vulcanus_crushing_basic.png"
+vulcanus_asteroid_chunk_crushing.order = "i[vulcanus].a[basic]"
+vulcanus_asteroid_chunk_crushing.enabled = false
+vulcanus_asteroid_chunk_crushing.energy_required = 2
+vulcanus_asteroid_chunk_crushing.ingredients = { { type = "item", name = "astra-vulcanic-asteroid-chunk", amount = 1 } }
+vulcanus_asteroid_chunk_crushing.results = { 
+    { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
+    { type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 } 
+}
+nauvis_asteroid_chunk_crushing.name = "astra-nauvis-asteroid-crushing"
+nauvis_asteroid_chunk_crushing.icon = "__Astra-Asteroids__/graphics/nauvis_crushing_basic.png"
+nauvis_asteroid_chunk_crushing.order = "h[nauvis].a[basic]"
+nauvis_asteroid_chunk_crushing.enabled = false
+nauvis_asteroid_chunk_crushing.energy_required = 2
+nauvis_asteroid_chunk_crushing.ingredients = { { type = "item", name = "astra-nauvis-asteroid-chunk", amount = 1 } }
+nauvis_asteroid_chunk_crushing.results = { 
+    { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
+    { type = "item", name = "uranium-ore", amount_min = 10, amount_max = 12, probability = 1 } 
+}
+gleba_asteroid_chunk_crushing.name = "astra-gleba-asteroid-crushing"
+gleba_asteroid_chunk_crushing.icon = "__Astra-Asteroids__/graphics/gleba_crushing_basic.png"
+gleba_asteroid_chunk_crushing.order = "j[gleba].a[basic]"
+gleba_asteroid_chunk_crushing.enabled = false
+gleba_asteroid_chunk_crushing.energy_required = 2
+gleba_asteroid_chunk_crushing.ingredients = { { type = "item", name = "astra-gleba-asteroid-chunk", amount = 1 } }
+gleba_asteroid_chunk_crushing.results = { 
+    { type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
+    { type = "item", name = "jellynut-seed", amount_min = 1, amount_max = 1, probability = 0.1 }, 
+    { type = "item", name = "spoilage", amount_min = 5, amount_max = 10, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
+    { type = "item", name = "yumako-seed", amount_min = 1, amount_max = 1, probability = 0.1 } 
+}
+fulgoran_asteroid_chunk_crushing.name = "astra-fulgoran-asteroid-crushing"
+fulgoran_asteroid_chunk_crushing.icon = "__Astra-Asteroids__/graphics/fulgora_crushing_basic.png"
+fulgoran_asteroid_chunk_crushing.order = "k[fulgora].a[basic]"
+fulgoran_asteroid_chunk_crushing.enabled = false
+fulgoran_asteroid_chunk_crushing.energy_required = 2
+fulgoran_asteroid_chunk_crushing.ingredients = { { type = "item", name = "astra-fulgoran-asteroid-chunk", amount = 1 } }
+fulgoran_asteroid_chunk_crushing.results = { 
+    { type = "item", name = "astra-fulgoran-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
+    { type = "item", name = "scrap", amount_min = 5, amount_max = 10, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 } 
+}
+aquilo-asteroid-chunk_crushing.name = "astra-aquilo-asteroid-crushing"
+aquilo-asteroid-chunk_crushing.icon = "__Astra-Asteroids__/graphics/crude_crushing_basic.png"
+aquilo-asteroid-chunk_crushing.order = "l[aquilo].a[basic]"
+aquilo-asteroid-chunk_crushing.enabled = false
+aquilo-asteroid-chunk_crushing.energy_required = 2
+aquilo-asteroid-chunk_crushing.ingredients = { { type = "item", name = "astra-aquilo-asteroid-chunk", amount = 1 } }
+aquilo-asteroid-chunk_crushing.results = { 
+    { type = "item", name = "astra-aquilo-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
+    { type = "item", name = "lithium", amount_min = 2, amount_max = 5, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+}
+vulcanis_asteroid_chunk_crushing_adv.name = "astra-advanced-vulcanis-asteroid-crushing"
+vulcanis_asteroid_chunk_crushing_adv.icon = "__Astra-Asteroids__/graphics/vulcanus_crushing_basic.png"
+vulcanis_asteroid_chunk_crushing_adv.order = "i[vulcanus].b[adv]"
+vulcanis_asteroid_chunk_crushing_adv.enabled = false
+vulcanis_asteroid_chunk_crushing_adv.energy_required = 5
+vulcanis_asteroid_chunk_crushing_adv.ingredients = { { type = "item", name = "astra-vulcanic-asteroid-chunk", amount = 1 } }
+vulcanis_asteroid_chunk_crushing_adv.results = { 
+    { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
+    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }, 
+    { type = "item", name = "tungsten-ore", amount_min = 10, amount_max = 14, probability = 1 } 
+}
+nauvis_asteroid_chunk_crushing_adv.name = "astra-advanced-nauvis-asteroid-crushing"
+nauvis_asteroid_chunk_crushing_adv.icon = "__Astra-Asteroids__/graphics/nauvis_crushing_basic.png"
+nauvis_asteroid_chunk_crushing_adv.order = "h[nauvis].b[adv]"
+nauvis_asteroid_chunk_crushing_adv.enabled = false
+nauvis_asteroid_chunk_crushing_adv.energy_required = 5
+nauvis_asteroid_chunk_crushing_adv.ingredients = { { type = "item", name = "astra-nauvis-asteroid-chunk", amount = 1 } }
+nauvis_asteroid_chunk_crushing_adv.results = { 
+    { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
+    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }, 
+    { type = "item", name = "uranium-235", amount_min = 1, amount_max = 1, probability = 0.3 }, 
+    { type = "item", name = "uranium-238", amount_min = 3, amount_max = 5, probability = 1 } 
+}
+gleba_asteroid_chunk_crushing_adv.name = "astra-advanced-gleba-asteroid-crushing"
+gleba_asteroid_chunk_crushing_adv.icon = "__Astra-Asteroids__/graphics/gleba_crushing_basic.png"
+gleba_asteroid_chunk_crushing_adv.order = "j[gleba].b[adv]"
+gleba_asteroid_chunk_crushing_adv.enabled = false
+gleba_asteroid_chunk_crushing_adv.energy_required = 5
+gleba_asteroid_chunk_crushing_adv.ingredients = { { type = "item", name = "astra-gleba-asteroid-chunk", amount = 1 } }
+gleba_asteroid_chunk_crushing_adv.results = { 
+    { type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
+    { type = "item", name = "jellynut-seed", amount_min = 1, amount_max = 2, probability = 0.3 }, 
+    { type = "item", name = "spoilage", amount_min = 10, amount_max = 20, probability = 1 }, 
+    { type = "item", name = "yumako-seed", amount_min = 1, amount_max = 2, probability = 0.3 } 
+}
+fulgoran_asteroid_chunk_crushing_adv.name = "astra-advanced-fulgoran-asteroid-crushing"
+fulgoran_asteroid_chunk_crushing_adv.icon = "__Astra-Asteroids__/graphics/fulgora_crushing_basic.png"
+fulgoran_asteroid_chunk_crushing_adv.order = "k[fulgora].b[adv]"
+fulgoran_asteroid_chunk_crushing_adv.enabled = false
+fulgoran_asteroid_chunk_crushing_adv.energy_required = 5
+fulgoran_asteroid_chunk_crushing_adv.ingredients = { { type = "item", name = "astra-fulgoran-asteroid-chunk", amount = 1 } }
+fulgoran_asteroid_chunk_crushing_adv.results = { 
+    { type = "item", name = "astra-fulgoran-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
+    { type = "item", name = "holmium-ore", amount_min = 1, amount_max = 2, probability = 0.4 }, 
+    { type = "item", name = "scrap", amount_min = 10, amount_max = 15, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 } 
+}
+crude_asteroid_chunk_crushing_adv.name = "astra-advanced-crude-asteroid-crushing"
+crude_asteroid_chunk_crushing_adv.icon = "__Astra-Asteroids__/graphics/crude_crushing_basic.png"
+crude_asteroid_chunk_crushing_adv.order = "g[crude].b[adv]"
+crude_asteroid_chunk_crushing_adv.enabled = false
+crude_asteroid_chunk_crushing_adv.energy_required = 5
+crude_asteroid_chunk_crushing_adv.ingredients = { { type = "item", name = "astra-crude-asteroid-chunk", amount = 1 } }
+crude_asteroid_chunk_crushing_adv.results = { 
+    { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
+    { type = "item", name = "astra-oilstone", amount_min = 5, amount_max = 8, probability = 1 }, 
+    { type = "item", name = "coal", amount_min = 5, amount_max = 8, probability = 1 } 
+}
+vulcanus_special_crushing.name = "astra-vulcanus-special-crushing"
+vulcanus_special_crushing.icon = "__Astra-Asteroids__/graphics/vulcanus_crushing_basic.png"
+vulcanus_special_crushing.order = "i[vulcanus].z[special]"
+vulcanus_special_crushing.enabled = false
+vulcanus_special_crushing.energy_required = 5
+vulcanus_special_crushing.ingredients = { { type = "item", name = "astra-vulcanic-asteroid-chunk", amount = 1 }, { type = "item", name = "metallic-astroid-chunk", amount = 1 } }
+vulcanus_special_crushing.results = { 
+    { type = "fluid", name = "lava", amount_min = 2000, amount_max = 2000, probability = 1 }, 
+    { type = "item", name = "tungsten-ore", amount_min = 12, amount_max = 12, probability = 1 } 
+}
+fulgoran_special_crushing.name = "astra-fulgoran-special-crushing"
+fulgoran_special_crushing.icon = "__Astra-Asteroids__/graphics/fulgora_crushing_basic.png"
+fulgoran_special_crushing.order = "k[fulgora].z[special]"
+fulgoran_special_crushing.enabled = false
+fulgoran_special_crushing.energy_required = 10
+fulgoran_special_crushing.ingredients = { { type = "item", name = "astra-fulgoran-asteroid-chunk", amount = 1 }, { type = "item", name = "carbonic-asteroid-chunk", amount = 1 } }
+fulgoran_special_crushing.results = { 
+    { type = "fluid", name = "heavy-oil", amount_min = 20, amount_max = 20, probability = 1 }, 
+    { type = "fluid", name = "holmium-solution", amount_min = 20, amount_max = 20, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+}</v>
       </c>
       <c r="G4" s="13" t="s">
         <v>193</v>
@@ -20685,13 +20862,11 @@
       <c r="AO8" s="14" t="str" cm="1">
         <f t="array" ref="AO8" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "ice", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
-    { type = "item", name = "iron-ore", amount_min = 20, amount_max = 20, probability = 1 }, 
-    { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
 }</v>
       </c>
       <c r="AP8" s="15" t="str" cm="1">
@@ -20707,9 +20882,7 @@
 .ingredients = { { type = "item", name = "oxide-asteroid-chunk", amount = 1 } }
 .results = { 
     { type = "item", name = "ice", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
-    { type = "item", name = "iron-ore", amount_min = 20, amount_max = 20, probability = 1 }, 
-    { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
 }</v>
       </c>
     </row>
@@ -20866,13 +21039,10 @@
       <c r="AO9" s="14" t="str" cm="1">
         <f t="array" ref="AO9" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
-    { type = "item", name = "iron-ore", amount_min = 20, amount_max = 20, probability = 1 }, 
-    { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
-    { type = "item", name = "astra-oilstone", amount_min = 4, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+    { type = "item", name = "iron-ore", amount_min = 20, amount_max = 20, probability = 1 } 
 }</v>
       </c>
       <c r="AP9" s="15" t="str" cm="1">
@@ -20887,10 +21057,7 @@
 .energy_required = 2
 .ingredients = { { type = "item", name = "metallic-astroid-chunk", amount = 1 } }
 .results = { 
-    { type = "item", name = "iron-ore", amount_min = 20, amount_max = 20, probability = 1 }, 
-    { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
-    { type = "item", name = "astra-oilstone", amount_min = 4, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+    { type = "item", name = "iron-ore", amount_min = 20, amount_max = 20, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -21050,13 +21217,12 @@
       <c r="AO10" s="14" t="str" cm="1">
         <f t="array" ref="AO10" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "astra-oilstone", amount_min = 4, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "carbon", amount_min = 10, amount_max = 10, probability = 1 } 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
 }</v>
       </c>
       <c r="AP10" s="15" t="str" cm="1">
@@ -21073,8 +21239,7 @@
 crude_asteroid_chunk_crushing.results = { 
     { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "astra-oilstone", amount_min = 4, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "carbon", amount_min = 10, amount_max = 10, probability = 1 } 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -21231,13 +21396,10 @@
       <c r="AO11" s="14" t="str" cm="1">
         <f t="array" ref="AO11" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
-    { type = "item", name = "carbon", amount_min = 10, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 } 
+    { type = "item", name = "carbon", amount_min = 10, amount_max = 10, probability = 1 } 
 }</v>
       </c>
       <c r="AP11" s="15" t="str" cm="1">
@@ -21252,10 +21414,7 @@
 .energy_required = 2
 .ingredients = { { type = "item", name = "carbonic-asteroid-chunk", amount = 1 } }
 .results = { 
-    { type = "item", name = "carbon", amount_min = 10, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 } 
+    { type = "item", name = "carbon", amount_min = 10, amount_max = 10, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -21415,13 +21574,12 @@
       <c r="AO12" s="14" t="str" cm="1">
         <f t="array" ref="AO12" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 } 
 }</v>
       </c>
       <c r="AP12" s="15" t="str" cm="1">
@@ -21438,8 +21596,7 @@
 vulcanus_asteroid_chunk_crushing.results = { 
     { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -21599,13 +21756,12 @@
       <c r="AO13" s="14" t="str" cm="1">
         <f t="array" ref="AO13" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "uranium-ore", amount_min = 10, amount_max = 12, probability = 1 }, 
-    { type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "uranium-ore", amount_min = 10, amount_max = 12, probability = 1 } 
 }</v>
       </c>
       <c r="AP13" s="15" t="str" cm="1">
@@ -21622,8 +21778,7 @@
 nauvis_asteroid_chunk_crushing.results = { 
     { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "uranium-ore", amount_min = 10, amount_max = 12, probability = 1 }, 
-    { type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "uranium-ore", amount_min = 10, amount_max = 12, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -21783,13 +21938,14 @@
       <c r="AO14" s="14" t="str" cm="1">
         <f t="array" ref="AO14" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "jellynut-seed", amount_min = 1, amount_max = 1, probability = 0.1 }, 
     { type = "item", name = "spoilage", amount_min = 5, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
+    { type = "item", name = "yumako-seed", amount_min = 1, amount_max = 1, probability = 0.1 } 
 }</v>
       </c>
       <c r="AP14" s="15" t="str" cm="1">
@@ -21807,7 +21963,8 @@
     { type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "jellynut-seed", amount_min = 1, amount_max = 1, probability = 0.1 }, 
     { type = "item", name = "spoilage", amount_min = 5, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
+    { type = "item", name = "yumako-seed", amount_min = 1, amount_max = 1, probability = 0.1 } 
 }</v>
       </c>
     </row>
@@ -21967,13 +22124,12 @@
       <c r="AO15" s="14" t="str" cm="1">
         <f t="array" ref="AO15" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-fulgoran-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "scrap", amount_min = 5, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }, 
-    { type = "item", name = "astra-aquilo-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 } 
 }</v>
       </c>
       <c r="AP15" s="15" t="str" cm="1">
@@ -21990,8 +22146,7 @@
 fulgoran_asteroid_chunk_crushing.results = { 
     { type = "item", name = "astra-fulgoran-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "scrap", amount_min = 5, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }, 
-    { type = "item", name = "astra-aquilo-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 } 
+    { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -22151,13 +22306,12 @@
       <c r="AO16" s="14" t="str" cm="1">
         <f t="array" ref="AO16" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-aquilo-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "lithium", amount_min = 2, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "calcite", amount_min = 2, amount_max = 2, probability = 1 } 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
 }</v>
       </c>
       <c r="AP16" s="15" t="str" cm="1">
@@ -22174,14 +22328,16 @@
 aquilo-asteroid-chunk_crushing.results = { 
     { type = "item", name = "astra-aquilo-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }, 
     { type = "item", name = "lithium", amount_min = 2, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }, 
-    { type = "item", name = "calcite", amount_min = 2, amount_max = 2, probability = 1 } 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
 }</v>
       </c>
     </row>
     <row r="17" spans="3:42" ht="18.75" customHeight="1">
       <c r="C17" t="s">
         <v>105</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="E17" s="2" t="b">
         <f>OR(ISNUMBER(SEARCH("Adv", Table7[[#This Row],[Recipe]])), ISNUMBER(SEARCH("Special", Table7[[#This Row],[Recipe]])))</f>
@@ -22329,13 +22485,12 @@
       <c r="AO17" s="14" t="str" cm="1">
         <f t="array" ref="AO17" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "calcite", amount_min = 2, amount_max = 2, probability = 1 }, 
     { type = "item", name = "ice", amount_min = 3, amount_max = 3, probability = 1 }, 
-    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
-    { type = "item", name = "copper-ore", amount_min = 4, amount_max = 4, probability = 1 } 
+    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
 }</v>
       </c>
       <c r="AP17" s="15" t="str" cm="1">
@@ -22352,14 +22507,16 @@
 .results = { 
     { type = "item", name = "calcite", amount_min = 2, amount_max = 2, probability = 1 }, 
     { type = "item", name = "ice", amount_min = 3, amount_max = 3, probability = 1 }, 
-    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
-    { type = "item", name = "copper-ore", amount_min = 4, amount_max = 4, probability = 1 } 
+    { type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
 }</v>
       </c>
     </row>
     <row r="18" spans="3:42" ht="18.75" customHeight="1">
       <c r="C18" t="s">
         <v>103</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="E18" s="2" t="b">
         <f>OR(ISNUMBER(SEARCH("Adv", Table7[[#This Row],[Recipe]])), ISNUMBER(SEARCH("Special", Table7[[#This Row],[Recipe]])))</f>
@@ -22507,13 +22664,12 @@
       <c r="AO18" s="14" t="str" cm="1">
         <f t="array" ref="AO18" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "copper-ore", amount_min = 4, amount_max = 4, probability = 1 }, 
     { type = "item", name = "iron-ore", amount_min = 10, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "metallic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
-    { type = "item", name = "carbon", amount_min = 5, amount_max = 5, probability = 1 } 
+    { type = "item", name = "metallic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
 }</v>
       </c>
       <c r="AP18" s="15" t="str" cm="1">
@@ -22530,14 +22686,16 @@
 .results = { 
     { type = "item", name = "copper-ore", amount_min = 4, amount_max = 4, probability = 1 }, 
     { type = "item", name = "iron-ore", amount_min = 10, amount_max = 10, probability = 1 }, 
-    { type = "item", name = "metallic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
-    { type = "item", name = "carbon", amount_min = 5, amount_max = 5, probability = 1 } 
+    { type = "item", name = "metallic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
 }</v>
       </c>
     </row>
     <row r="19" spans="3:42" ht="18.75" customHeight="1">
       <c r="C19" t="s">
         <v>104</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="E19" s="2" t="b">
         <f>OR(ISNUMBER(SEARCH("Adv", Table7[[#This Row],[Recipe]])), ISNUMBER(SEARCH("Special", Table7[[#This Row],[Recipe]])))</f>
@@ -22685,13 +22843,12 @@
       <c r="AO19" s="14" t="str" cm="1">
         <f t="array" ref="AO19" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "carbon", amount_min = 5, amount_max = 5, probability = 1 }, 
     { type = "item", name = "carbonic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
-    { type = "item", name = "sulfur", amount_min = 2, amount_max = 2, probability = 1 }, 
-    { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
+    { type = "item", name = "sulfur", amount_min = 2, amount_max = 2, probability = 1 } 
 }</v>
       </c>
       <c r="AP19" s="15" t="str" cm="1">
@@ -22708,8 +22865,7 @@
 .results = { 
     { type = "item", name = "carbon", amount_min = 5, amount_max = 5, probability = 1 }, 
     { type = "item", name = "carbonic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
-    { type = "item", name = "sulfur", amount_min = 2, amount_max = 2, probability = 1 }, 
-    { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
+    { type = "item", name = "sulfur", amount_min = 2, amount_max = 2, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -22869,13 +23025,12 @@
       <c r="AO20" s="14" t="str" cm="1">
         <f t="array" ref="AO20" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
     { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 10, amount_max = 14, probability = 1 }, 
-    { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
+    { type = "item", name = "tungsten-ore", amount_min = 10, amount_max = 14, probability = 1 } 
 }</v>
       </c>
       <c r="AP20" s="15" t="str" cm="1">
@@ -22892,8 +23047,7 @@
 vulcanis_asteroid_chunk_crushing_adv.results = { 
     { type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
     { type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 10, amount_max = 14, probability = 1 }, 
-    { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 } 
+    { type = "item", name = "tungsten-ore", amount_min = 10, amount_max = 14, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -23053,7 +23207,7 @@
       <c r="AO21" s="14" t="str" cm="1">
         <f t="array" ref="AO21" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
@@ -23237,7 +23391,7 @@
       <c r="AO22" s="14" t="str" cm="1">
         <f t="array" ref="AO22" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
@@ -23421,7 +23575,7 @@
       <c r="AO23" s="14" t="str" cm="1">
         <f t="array" ref="AO23" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-fulgoran-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
@@ -23605,13 +23759,12 @@
       <c r="AO24" s="14" t="str" cm="1">
         <f t="array" ref="AO24" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
     { type = "item", name = "astra-oilstone", amount_min = 5, amount_max = 8, probability = 1 }, 
-    { type = "item", name = "coal", amount_min = 5, amount_max = 8, probability = 1 }, 
-    { type = "fluid", name = "lava", amount_min = 2000, amount_max = 2000, probability = 1 } 
+    { type = "item", name = "coal", amount_min = 5, amount_max = 8, probability = 1 } 
 }</v>
       </c>
       <c r="AP24" s="15" t="str" cm="1">
@@ -23628,8 +23781,7 @@
 crude_asteroid_chunk_crushing_adv.results = { 
     { type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }, 
     { type = "item", name = "astra-oilstone", amount_min = 5, amount_max = 8, probability = 1 }, 
-    { type = "item", name = "coal", amount_min = 5, amount_max = 8, probability = 1 }, 
-    { type = "fluid", name = "lava", amount_min = 2000, amount_max = 2000, probability = 1 } 
+    { type = "item", name = "coal", amount_min = 5, amount_max = 8, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -23794,13 +23946,11 @@
       <c r="AO25" s="14" t="str" cm="1">
         <f t="array" ref="AO25" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
         <v>{ 
     { type = "fluid", name = "lava", amount_min = 2000, amount_max = 2000, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 12, amount_max = 12, probability = 1 }, 
-    { type = "fluid", name = "heavy-oil", amount_min = 20, amount_max = 20, probability = 1 }, 
-    { type = "fluid", name = "holmium-solution", amount_min = 20, amount_max = 20, probability = 1 } 
+    { type = "item", name = "tungsten-ore", amount_min = 12, amount_max = 12, probability = 1 } 
 }</v>
       </c>
       <c r="AP25" s="15" t="str" cm="1">
@@ -23816,9 +23966,7 @@
 vulcanus_special_crushing.ingredients = { { type = "item", name = "astra-vulcanic-asteroid-chunk", amount = 1 }, { type = "item", name = "metallic-astroid-chunk", amount = 1 } }
 vulcanus_special_crushing.results = { 
     { type = "fluid", name = "lava", amount_min = 2000, amount_max = 2000, probability = 1 }, 
-    { type = "item", name = "tungsten-ore", amount_min = 12, amount_max = 12, probability = 1 }, 
-    { type = "fluid", name = "heavy-oil", amount_min = 20, amount_max = 20, probability = 1 }, 
-    { type = "fluid", name = "holmium-solution", amount_min = 20, amount_max = 20, probability = 1 } 
+    { type = "item", name = "tungsten-ore", amount_min = 12, amount_max = 12, probability = 1 } 
 }</v>
       </c>
     </row>
@@ -23978,19 +24126,19 @@
 &amp; " }"</f>
         <v>{ { type = "item", name = "astra-nauvis-asteroid-chunk", amount = 1 } }</v>
       </c>
-      <c r="AO26" s="14" t="e" cm="1">
+      <c r="AO26" s="14" t="e" cm="1" vm="2">
         <f t="array" ref="AO26" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AP26" s="15" t="e" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="AP26" s="15" t="e" cm="1" vm="3">
         <f t="array" ref="AP26">_xlfn.TEXTJOIN("
 ", TRUE, Table7[[#This Row],[Variable''s Name]] &amp; "." &amp; Table7[[#Headers],[name]:[energy_required]] &amp; " = " &amp; Table7[[#This Row],[name]:[energy_required]]) &amp; "
 " &amp; Table7[[#This Row],[Variable''s Name]] &amp; ".ingredients = " &amp; Table7[[#This Row],[Ingredient String]] &amp; "
 " &amp; Table7[[#This Row],[Variable''s Name]] &amp; ".results = " &amp; Table7[[#This Row],[Results String]]</f>
-        <v>#N/A</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="27" spans="3:42" ht="18.75" customHeight="1">
@@ -24149,19 +24297,19 @@
 &amp; " }"</f>
         <v>{ { type = "item", name = "astra-gleba-asteroid-chunk", amount = 1 } }</v>
       </c>
-      <c r="AO27" s="14" t="e" cm="1">
+      <c r="AO27" s="14" t="e" cm="1" vm="2">
         <f t="array" ref="AO27" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AP27" s="15" t="e" cm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="AP27" s="15" t="e" cm="1" vm="3">
         <f t="array" ref="AP27">_xlfn.TEXTJOIN("
 ", TRUE, Table7[[#This Row],[Variable''s Name]] &amp; "." &amp; Table7[[#Headers],[name]:[energy_required]] &amp; " = " &amp; Table7[[#This Row],[name]:[energy_required]]) &amp; "
 " &amp; Table7[[#This Row],[Variable''s Name]] &amp; ".ingredients = " &amp; Table7[[#This Row],[Ingredient String]] &amp; "
 " &amp; Table7[[#This Row],[Variable''s Name]] &amp; ".results = " &amp; Table7[[#This Row],[Results String]]</f>
-        <v>#N/A</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="28" spans="3:42" ht="23.25" customHeight="1">
@@ -24322,19 +24470,33 @@
 &amp; " }"</f>
         <v>{ { type = "item", name = "astra-fulgoran-asteroid-chunk", amount = 1 }, { type = "item", name = "carbonic-asteroid-chunk", amount = 1 } }</v>
       </c>
-      <c r="AO28" s="14" t="e" cm="1">
+      <c r="AO28" s="14" t="str" cm="1">
         <f t="array" ref="AO28" xml:space="preserve"> "{ 
     " &amp; _xlfn.TEXTJOIN(", 
-    ", TRUE, _xlfn._xlws.FILTER(Table7[[#This Row],[Results 1]:[Results 4]], IFERROR(--Table7[[#This Row],[Results 1]:[Results 4]], TRUE))) &amp; " 
+    ", TRUE, _xlfn._xlws.FILTER(Table8[string], Table8[Recipe] = Table7[[#This Row],[Recipe]])) &amp; " 
 }"</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AP28" s="15" t="e" cm="1">
+        <v>{ 
+    { type = "fluid", name = "heavy-oil", amount_min = 20, amount_max = 20, probability = 1 }, 
+    { type = "fluid", name = "holmium-solution", amount_min = 20, amount_max = 20, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+}</v>
+      </c>
+      <c r="AP28" s="15" t="str" cm="1">
         <f t="array" ref="AP28">_xlfn.TEXTJOIN("
 ", TRUE, Table7[[#This Row],[Variable''s Name]] &amp; "." &amp; Table7[[#Headers],[name]:[energy_required]] &amp; " = " &amp; Table7[[#This Row],[name]:[energy_required]]) &amp; "
 " &amp; Table7[[#This Row],[Variable''s Name]] &amp; ".ingredients = " &amp; Table7[[#This Row],[Ingredient String]] &amp; "
 " &amp; Table7[[#This Row],[Variable''s Name]] &amp; ".results = " &amp; Table7[[#This Row],[Results String]]</f>
-        <v>#REF!</v>
+        <v>fulgoran_special_crushing.name = "astra-fulgoran-special-crushing"
+fulgoran_special_crushing.icon = "__Astra-Asteroids__/graphics/fulgora_crushing_basic.png"
+fulgoran_special_crushing.order = "k[fulgora].z[special]"
+fulgoran_special_crushing.enabled = false
+fulgoran_special_crushing.energy_required = 10
+fulgoran_special_crushing.ingredients = { { type = "item", name = "astra-fulgoran-asteroid-chunk", amount = 1 }, { type = "item", name = "carbonic-asteroid-chunk", amount = 1 } }
+fulgoran_special_crushing.results = { 
+    { type = "fluid", name = "heavy-oil", amount_min = 20, amount_max = 20, probability = 1 }, 
+    { type = "fluid", name = "holmium-solution", amount_min = 20, amount_max = 20, probability = 1 }, 
+    { type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 } 
+}</v>
       </c>
     </row>
     <row r="32" spans="3:42">
@@ -26460,17 +26622,17 @@
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C8:E28 AP8:AP28 F13:AE13 AF13:AM15 F14:Y14 AA14:AE14 F15:AE15 F16:AM18 E19:Y19 AE19:AM19 F20:AM27 F8:AM12">
-    <cfRule type="expression" dxfId="16" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>LEN($D8) &gt; 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28">
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>LEN($D28) &gt; 0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I28">
-    <cfRule type="expression" dxfId="21" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>LEN($D28) &gt; 0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26483,7 +26645,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0CAC3E1-19B2-497F-BF02-30D86B7FD830}">
-  <dimension ref="B3:K59"/>
+  <dimension ref="B3:L59"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3.75" customWidth="1"/>
@@ -26491,6 +26653,7 @@
     <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.375" bestFit="1" customWidth="1"/>
     <col min="5" max="10" width="10.375" customWidth="1"/>
+    <col min="12" max="12" width="34" customWidth="1"/>
     <col min="15" max="15" width="31.5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25.625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="25.375" bestFit="1" customWidth="1"/>
@@ -26524,7 +26687,7 @@
     <col min="47" max="47" width="11.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:11" s="14" customFormat="1" ht="54" customHeight="1">
+    <row r="3" spans="2:12" s="14" customFormat="1" ht="54" customHeight="1">
       <c r="B3" s="15" t="s">
         <v>23</v>
       </c>
@@ -26555,8 +26718,11 @@
       <c r="K3" s="15" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="4" spans="2:11">
+      <c r="L3" s="15" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12">
       <c r="B4" s="2" t="s">
         <v>102</v>
       </c>
@@ -26591,8 +26757,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.4</v>
       </c>
-    </row>
-    <row r="5" spans="2:11">
+      <c r="L4" s="25" t="str" cm="1">
+        <f t="array" ref="L4">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "ice", amount_min = 5, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12">
       <c r="B5" s="2" t="s">
         <v>102</v>
       </c>
@@ -26627,8 +26801,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="2:11">
+      <c r="L5" s="25" t="str" cm="1">
+        <f t="array" ref="L5">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12">
       <c r="B6" s="2" t="s">
         <v>351</v>
       </c>
@@ -26663,8 +26845,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="7" spans="2:11">
+      <c r="L6" s="25" t="str" cm="1">
+        <f t="array" ref="L6">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "iron-ore", amount_min = 20, amount_max = 20, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12">
       <c r="B7" s="2" t="s">
         <v>49</v>
       </c>
@@ -26699,8 +26889,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="2:11">
+      <c r="L7" s="25" t="str" cm="1">
+        <f t="array" ref="L7">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12">
       <c r="B8" s="2" t="s">
         <v>49</v>
       </c>
@@ -26735,8 +26933,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.44444444444444442</v>
       </c>
-    </row>
-    <row r="9" spans="2:11">
+      <c r="L8" s="25" t="str" cm="1">
+        <f t="array" ref="L8">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-oilstone", amount_min = 4, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12">
       <c r="B9" s="2" t="s">
         <v>49</v>
       </c>
@@ -26771,8 +26977,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.4</v>
       </c>
-    </row>
-    <row r="10" spans="2:11">
+      <c r="L9" s="25" t="str" cm="1">
+        <f t="array" ref="L9">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12">
       <c r="B10" s="2" t="s">
         <v>352</v>
       </c>
@@ -26807,8 +27021,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.2</v>
       </c>
-    </row>
-    <row r="11" spans="2:11">
+      <c r="L10" s="25" t="str" cm="1">
+        <f t="array" ref="L10">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "carbon", amount_min = 10, amount_max = 10, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12">
       <c r="B11" s="2" t="s">
         <v>50</v>
       </c>
@@ -26843,8 +27065,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="2:11">
+      <c r="L11" s="25" t="str" cm="1">
+        <f t="array" ref="L11">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12">
       <c r="B12" s="2" t="s">
         <v>50</v>
       </c>
@@ -26879,8 +27109,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.4</v>
       </c>
-    </row>
-    <row r="13" spans="2:11">
+      <c r="L12" s="25" t="str" cm="1">
+        <f t="array" ref="L12">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12">
       <c r="B13" s="2" t="s">
         <v>50</v>
       </c>
@@ -26915,8 +27153,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.44444444444444442</v>
       </c>
-    </row>
-    <row r="14" spans="2:11">
+      <c r="L13" s="25" t="str" cm="1">
+        <f t="array" ref="L13">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "tungsten-ore", amount_min = 4, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12">
       <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
@@ -26951,8 +27197,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="2:11">
+      <c r="L14" s="25" t="str" cm="1">
+        <f t="array" ref="L14">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12">
       <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
@@ -26987,8 +27241,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.4</v>
       </c>
-    </row>
-    <row r="16" spans="2:11">
+      <c r="L15" s="25" t="str" cm="1">
+        <f t="array" ref="L15">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12">
       <c r="B16" s="2" t="s">
         <v>40</v>
       </c>
@@ -27023,8 +27285,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.18181818181818182</v>
       </c>
-    </row>
-    <row r="17" spans="2:11">
+      <c r="L16" s="25" t="str" cm="1">
+        <f t="array" ref="L16">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "uranium-ore", amount_min = 10, amount_max = 12, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12">
       <c r="B17" s="2" t="s">
         <v>52</v>
       </c>
@@ -27059,8 +27329,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="2:11">
+      <c r="L17" s="25" t="str" cm="1">
+        <f t="array" ref="L17">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12">
       <c r="B18" s="2" t="s">
         <v>52</v>
       </c>
@@ -27095,8 +27373,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="2:11">
+      <c r="L18" s="25" t="str" cm="1">
+        <f t="array" ref="L18">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "jellynut-seed", amount_min = 1, amount_max = 1, probability = 0.1 }</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12">
       <c r="B19" s="2" t="s">
         <v>52</v>
       </c>
@@ -27131,8 +27417,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.26666666666666666</v>
       </c>
-    </row>
-    <row r="20" spans="2:11">
+      <c r="L19" s="25" t="str" cm="1">
+        <f t="array" ref="L19">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "spoilage", amount_min = 5, amount_max = 10, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12">
       <c r="B20" s="2" t="s">
         <v>52</v>
       </c>
@@ -27167,8 +27461,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.4</v>
       </c>
-    </row>
-    <row r="21" spans="2:11">
+      <c r="L20" s="25" t="str" cm="1">
+        <f t="array" ref="L20">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12">
       <c r="B21" s="2" t="s">
         <v>52</v>
       </c>
@@ -27203,8 +27505,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="2:11">
+      <c r="L21" s="25" t="str" cm="1">
+        <f t="array" ref="L21">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "yumako-seed", amount_min = 1, amount_max = 1, probability = 0.1 }</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12">
       <c r="B22" s="2" t="s">
         <v>51</v>
       </c>
@@ -27239,8 +27549,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="23" spans="2:11">
+      <c r="L22" s="25" t="str" cm="1">
+        <f t="array" ref="L22">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-fulgoran-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12">
       <c r="B23" s="2" t="s">
         <v>51</v>
       </c>
@@ -27275,8 +27593,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.26666666666666666</v>
       </c>
-    </row>
-    <row r="24" spans="2:11">
+      <c r="L23" s="25" t="str" cm="1">
+        <f t="array" ref="L23">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "scrap", amount_min = 5, amount_max = 10, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12">
       <c r="B24" s="2" t="s">
         <v>51</v>
       </c>
@@ -27311,8 +27637,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="2:11">
+      <c r="L24" s="25" t="str" cm="1">
+        <f t="array" ref="L24">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12">
       <c r="B25" s="2" t="s">
         <v>340</v>
       </c>
@@ -27347,8 +27681,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="26" spans="2:11">
+      <c r="L25" s="25" t="str" cm="1">
+        <f t="array" ref="L25">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-aquilo-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.2 }</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12">
       <c r="B26" s="2" t="s">
         <v>340</v>
       </c>
@@ -27383,8 +27725,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.5714285714285714</v>
       </c>
-    </row>
-    <row r="27" spans="2:11">
+      <c r="L26" s="25" t="str" cm="1">
+        <f t="array" ref="L26">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "lithium", amount_min = 2, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12">
       <c r="B27" s="2" t="s">
         <v>340</v>
       </c>
@@ -27419,8 +27769,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.4</v>
       </c>
-    </row>
-    <row r="28" spans="2:11">
+      <c r="L27" s="25" t="str" cm="1">
+        <f t="array" ref="L27">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12">
       <c r="B28" s="2" t="s">
         <v>105</v>
       </c>
@@ -27455,8 +27813,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>2.5</v>
       </c>
-    </row>
-    <row r="29" spans="2:11">
+      <c r="L28" s="25" t="str" cm="1">
+        <f t="array" ref="L28">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "calcite", amount_min = 2, amount_max = 2, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12">
       <c r="B29" s="2" t="s">
         <v>105</v>
       </c>
@@ -27491,8 +27857,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>1.6666666666666667</v>
       </c>
-    </row>
-    <row r="30" spans="2:11">
+      <c r="L29" s="25" t="str" cm="1">
+        <f t="array" ref="L29">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "ice", amount_min = 3, amount_max = 3, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12">
       <c r="B30" s="2" t="s">
         <v>105</v>
       </c>
@@ -27527,8 +27901,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="31" spans="2:11">
+      <c r="L30" s="25" t="str" cm="1">
+        <f t="array" ref="L30">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "oxide-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12">
       <c r="B31" s="2" t="s">
         <v>103</v>
       </c>
@@ -27563,8 +27945,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>1.25</v>
       </c>
-    </row>
-    <row r="32" spans="2:11">
+      <c r="L31" s="25" t="str" cm="1">
+        <f t="array" ref="L31">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "copper-ore", amount_min = 4, amount_max = 4, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12">
       <c r="B32" s="2" t="s">
         <v>103</v>
       </c>
@@ -27599,8 +27989,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.5</v>
       </c>
-    </row>
-    <row r="33" spans="2:11">
+      <c r="L32" s="25" t="str" cm="1">
+        <f t="array" ref="L32">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "iron-ore", amount_min = 10, amount_max = 10, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12">
       <c r="B33" s="2" t="s">
         <v>103</v>
       </c>
@@ -27635,8 +28033,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="34" spans="2:11">
+      <c r="L33" s="25" t="str" cm="1">
+        <f t="array" ref="L33">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "metallic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12">
       <c r="B34" s="2" t="s">
         <v>104</v>
       </c>
@@ -27671,8 +28077,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="2:11">
+      <c r="L34" s="25" t="str" cm="1">
+        <f t="array" ref="L34">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "carbon", amount_min = 5, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12">
       <c r="B35" s="2" t="s">
         <v>104</v>
       </c>
@@ -27707,8 +28121,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="36" spans="2:11">
+      <c r="L35" s="25" t="str" cm="1">
+        <f t="array" ref="L35">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "carbonic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12">
       <c r="B36" s="2" t="s">
         <v>104</v>
       </c>
@@ -27743,8 +28165,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>2.5</v>
       </c>
-    </row>
-    <row r="37" spans="2:11">
+      <c r="L36" s="25" t="str" cm="1">
+        <f t="array" ref="L36">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "sulfur", amount_min = 2, amount_max = 2, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12">
       <c r="B37" s="2" t="s">
         <v>160</v>
       </c>
@@ -27779,8 +28209,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="38" spans="2:11">
+      <c r="L37" s="25" t="str" cm="1">
+        <f t="array" ref="L37">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-vulcanic-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12">
       <c r="B38" s="2" t="s">
         <v>160</v>
       </c>
@@ -27815,8 +28253,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="2:11">
+      <c r="L38" s="25" t="str" cm="1">
+        <f t="array" ref="L38">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12">
       <c r="B39" s="2" t="s">
         <v>160</v>
       </c>
@@ -27851,8 +28297,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.41666666666666669</v>
       </c>
-    </row>
-    <row r="40" spans="2:11">
+      <c r="L39" s="25" t="str" cm="1">
+        <f t="array" ref="L39">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "tungsten-ore", amount_min = 10, amount_max = 14, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="40" spans="2:12">
       <c r="B40" s="2" t="s">
         <v>46</v>
       </c>
@@ -27887,8 +28341,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="41" spans="2:11">
+      <c r="L40" s="25" t="str" cm="1">
+        <f t="array" ref="L40">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-nauvis-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12">
       <c r="B41" s="2" t="s">
         <v>46</v>
       </c>
@@ -27923,8 +28385,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="2:11">
+      <c r="L41" s="25" t="str" cm="1">
+        <f t="array" ref="L41">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12">
       <c r="B42" s="2" t="s">
         <v>46</v>
       </c>
@@ -27959,8 +28429,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>16.666666666666668</v>
       </c>
-    </row>
-    <row r="43" spans="2:11">
+      <c r="L42" s="25" t="str" cm="1">
+        <f t="array" ref="L42">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "uranium-235", amount_min = 1, amount_max = 1, probability = 0.3 }</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12">
       <c r="B43" s="2" t="s">
         <v>46</v>
       </c>
@@ -27995,8 +28473,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>1.25</v>
       </c>
-    </row>
-    <row r="44" spans="2:11">
+      <c r="L43" s="25" t="str" cm="1">
+        <f t="array" ref="L43">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "uranium-238", amount_min = 3, amount_max = 5, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="44" spans="2:12">
       <c r="B44" s="2" t="s">
         <v>161</v>
       </c>
@@ -28031,8 +28517,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="45" spans="2:11">
+      <c r="L44" s="25" t="str" cm="1">
+        <f t="array" ref="L44">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-gleba-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12">
       <c r="B45" s="2" t="s">
         <v>161</v>
       </c>
@@ -28067,8 +28561,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>11.111111111111111</v>
       </c>
-    </row>
-    <row r="46" spans="2:11">
+      <c r="L45" s="25" t="str" cm="1">
+        <f t="array" ref="L45">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "jellynut-seed", amount_min = 1, amount_max = 2, probability = 0.3 }</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12">
       <c r="B46" s="2" t="s">
         <v>161</v>
       </c>
@@ -28103,8 +28605,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.33333333333333331</v>
       </c>
-    </row>
-    <row r="47" spans="2:11">
+      <c r="L46" s="25" t="str" cm="1">
+        <f t="array" ref="L46">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "spoilage", amount_min = 10, amount_max = 20, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="47" spans="2:12">
       <c r="B47" s="2" t="s">
         <v>161</v>
       </c>
@@ -28139,8 +28649,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>11.111111111111111</v>
       </c>
-    </row>
-    <row r="48" spans="2:11">
+      <c r="L47" s="25" t="str" cm="1">
+        <f t="array" ref="L47">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "yumako-seed", amount_min = 1, amount_max = 2, probability = 0.3 }</v>
+      </c>
+    </row>
+    <row r="48" spans="2:12">
       <c r="B48" s="2" t="s">
         <v>162</v>
       </c>
@@ -28175,8 +28693,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="49" spans="2:11">
+      <c r="L48" s="25" t="str" cm="1">
+        <f t="array" ref="L48">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-fulgoran-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="49" spans="2:12">
       <c r="B49" s="2" t="s">
         <v>162</v>
       </c>
@@ -28211,8 +28737,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>8.3333333333333321</v>
       </c>
-    </row>
-    <row r="50" spans="2:11">
+      <c r="L49" s="25" t="str" cm="1">
+        <f t="array" ref="L49">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "holmium-ore", amount_min = 1, amount_max = 2, probability = 0.4 }</v>
+      </c>
+    </row>
+    <row r="50" spans="2:12">
       <c r="B50" s="2" t="s">
         <v>162</v>
       </c>
@@ -28247,8 +28781,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.4</v>
       </c>
-    </row>
-    <row r="51" spans="2:11">
+      <c r="L50" s="25" t="str" cm="1">
+        <f t="array" ref="L50">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "scrap", amount_min = 10, amount_max = 15, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="51" spans="2:12">
       <c r="B51" s="2" t="s">
         <v>162</v>
       </c>
@@ -28283,8 +28825,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="2:11">
+      <c r="L51" s="25" t="str" cm="1">
+        <f t="array" ref="L51">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 0, amount_max = 0, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="52" spans="2:12">
       <c r="B52" s="2" t="s">
         <v>233</v>
       </c>
@@ -28319,8 +28869,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="53" spans="2:11">
+      <c r="L52" s="25" t="str" cm="1">
+        <f t="array" ref="L52">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-crude-asteroid-chunk", amount_min = 1, amount_max = 1, probability = 0.05 }</v>
+      </c>
+    </row>
+    <row r="53" spans="2:12">
       <c r="B53" s="2" t="s">
         <v>233</v>
       </c>
@@ -28355,8 +28913,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.76923076923076916</v>
       </c>
-    </row>
-    <row r="54" spans="2:11">
+      <c r="L53" s="25" t="str" cm="1">
+        <f t="array" ref="L53">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "astra-oilstone", amount_min = 5, amount_max = 8, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="54" spans="2:12">
       <c r="B54" s="2" t="s">
         <v>233</v>
       </c>
@@ -28391,8 +28957,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.76923076923076916</v>
       </c>
-    </row>
-    <row r="55" spans="2:11">
+      <c r="L54" s="25" t="str" cm="1">
+        <f t="array" ref="L54">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "coal", amount_min = 5, amount_max = 8, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="55" spans="2:12">
       <c r="B55" s="2" t="s">
         <v>166</v>
       </c>
@@ -28427,8 +29001,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>2.5000000000000001E-3</v>
       </c>
-    </row>
-    <row r="56" spans="2:11">
+      <c r="L55" s="25" t="str" cm="1">
+        <f t="array" ref="L55">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "fluid", name = "lava", amount_min = 2000, amount_max = 2000, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="56" spans="2:12">
       <c r="B56" s="2" t="s">
         <v>166</v>
       </c>
@@ -28463,8 +29045,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.41666666666666669</v>
       </c>
-    </row>
-    <row r="57" spans="2:11">
+      <c r="L56" s="25" t="str" cm="1">
+        <f t="array" ref="L56">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "tungsten-ore", amount_min = 12, amount_max = 12, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="57" spans="2:12">
       <c r="B57" s="2" t="s">
         <v>164</v>
       </c>
@@ -28499,8 +29089,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.5</v>
       </c>
-    </row>
-    <row r="58" spans="2:11">
+      <c r="L57" s="25" t="str" cm="1">
+        <f t="array" ref="L57">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "fluid", name = "heavy-oil", amount_min = 20, amount_max = 20, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="58" spans="2:12">
       <c r="B58" s="2" t="s">
         <v>164</v>
       </c>
@@ -28535,8 +29133,16 @@
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>0.5</v>
       </c>
-    </row>
-    <row r="59" spans="2:11">
+      <c r="L58" s="25" t="str" cm="1">
+        <f t="array" ref="L58">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "fluid", name = "holmium-solution", amount_min = 20, amount_max = 20, probability = 1 }</v>
+      </c>
+    </row>
+    <row r="59" spans="2:12">
       <c r="B59" s="2" t="s">
         <v>164</v>
       </c>
@@ -28570,6 +29176,14 @@
       <c r="K59" s="2">
         <f>IFERROR(1/Table8[[#This Row],[EV/s]], 0)</f>
         <v>2</v>
+      </c>
+      <c r="L59" s="25" t="str" cm="1">
+        <f t="array" ref="L59">"{ " &amp;
+_xlfn.TEXTJOIN(", ",
+          TRUE,
+          {"type","name","amount_min","amount_max","probability"} &amp; " = " &amp; IF(NOT(ISNUMBER(Table8[[#This Row],[type]:[P]])), """" &amp; Table8[[#This Row],[type]:[P]] &amp; """", Table8[[#This Row],[type]:[P]]) ) &amp;
+" }"</f>
+        <v>{ type = "item", name = "stone", amount_min = 5, amount_max = 5, probability = 1 }</v>
       </c>
     </row>
   </sheetData>

</xml_diff>